<commit_message>
fix(gold): tipo = file_type puro (padrao consistente entre cursos)
Bug: tipo_of preferia keyword do nome antes do file_type -> 'ProvasIndutivas'
(demonstracao matematica) e 'provas.thy' (Isabelle) viravam tipo='prova' (exame).
Em MF "prova"=proof. O manifest ja estava certo (provas.thy=code,
ProvasIndutivas=material-de-aula); a cascata de keyword no gerador sobrescrevia.

Fix: tipo_of retorna file_type (pdf/codigo/imagem/link/material). Consistente
entre cursos (todos os PDFs = 'pdf'), sem misfire de keyword. Distincao semantica
(exercicio/prova) mora no nome+topico, nao no tipo. _TIPO_ORDER atualizado.

Regenerados MF/SO/TCC (nao rotulados). IA/ES2 committed mantem tipo antigo
(cosmetico, nao lido pelo crosswalk; regenerar exigiria re-rotular).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRQpbp1NNFwNrJaHsq41XT
</commit_message>
<xml_diff>
--- a/docs/reports/gold_templates/gold_MF_rotular.xlsx
+++ b/docs/reports/gold_templates/gold_MF_rotular.xlsx
@@ -498,17 +498,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>provas.thy</t>
+          <t>ConjuntosIndutivos.pdf</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>provas</t>
+          <t>Conjuntos Indutivos</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
@@ -521,17 +521,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>ProvasIndutivas_EspecificaçõesRecursivas.pdf</t>
+          <t>CorrecaoTerminacao.pdf</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Provas Indutivas Especificações Recursivas</t>
+          <t>Correcao Terminacao</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
@@ -544,17 +544,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>ProvasIndutivas_EspecificaçõesRecursivas_Arvores.pdf</t>
+          <t>ExerciciosConjuntosIndutivos.pdf</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Provas Indutivas Especificações Recursivas Arvores</t>
+          <t>Exercicios Conjuntos Indutivos</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
@@ -567,17 +567,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ProvasIndutivas_EspecificaçõesRecursivas_Listas.pdf</t>
+          <t>ExerciciosCorrecaoInducaoMatematica.pdf</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Provas Indutivas Especificações Recursivas Listas</t>
+          <t>Exercicios Correcao Inducao Matematica</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
@@ -590,17 +590,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>revisao_p1.pdf</t>
+          <t>ExerciciosCorrecaoTerminacao.pdf</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>revisao p1</t>
+          <t>Exercicios Correcao Terminacao</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
@@ -613,17 +613,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>revisao_p1_gabarito.pdf</t>
+          <t>ExerciciosDafny1.pdf</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>prova</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>revisao p1 gabarito</t>
+          <t>Exercicios Dafny1</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
@@ -636,17 +636,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosConjuntosIndutivos.pdf</t>
+          <t>ExerciciosDafny2.pdf</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Conjuntos Indutivos</t>
+          <t>Exercicios Dafny2</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
@@ -659,17 +659,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosCorrecaoInducaoMatematica.pdf</t>
+          <t>ExerciciosDafny3.pdf</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Correcao Inducao Matematica</t>
+          <t>Exercicios Dafny3</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
@@ -682,17 +682,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosCorrecaoTerminacao.pdf</t>
+          <t>ExerciciosDafny4.pdf</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Correcao Terminacao</t>
+          <t>Exercicios Dafny4</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr"/>
@@ -705,17 +705,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosDafny1.pdf</t>
+          <t>ExerciciosDafny5.pdf</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Dafny1</t>
+          <t>Exercicios Dafny5</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr"/>
@@ -728,17 +728,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosDafny2.pdf</t>
+          <t>ExerciciosEspecificacao.pdf</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Dafny2</t>
+          <t>Exercicios Especificacao</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr"/>
@@ -751,17 +751,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosDafny3.pdf</t>
+          <t>ExerciciosEspecificacao_respostas.pdf</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Dafny3</t>
+          <t>Exercicios Especificacao respostas</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
@@ -774,17 +774,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosDafny4.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosInvariantes.pdf</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Dafny4</t>
+          <t>Exercicios Formalizacao Algoritmos Invariantes</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr"/>
@@ -797,17 +797,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosDafny5.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosRecursao.pdf</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Dafny5</t>
+          <t>Exercicios Formalizacao Algoritmos Recursao</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr"/>
@@ -820,17 +820,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosEspecificacao.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosRecursao_respostas.pdf</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Especificacao</t>
+          <t>Exercicios Formalizacao Algoritmos Recursao respostas</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr"/>
@@ -843,17 +843,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosInvariantes.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosRecursao2.pdf</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Invariantes</t>
+          <t>Exercicios Formalizacao Algoritmos Recursao2</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr"/>
@@ -866,17 +866,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosRecursao.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosRecursao3.pdf</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Recursao</t>
+          <t>Exercicios Formalizacao Algoritmos Recursao3</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr"/>
@@ -889,17 +889,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosRecursao2.pdf</t>
+          <t>ExerciciosFormalizacaoAlgoritmosRecursao3_respostas.pdf</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Recursao2</t>
+          <t>Exercicios Formalizacao Algoritmos Recursao3 respostas</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr"/>
@@ -912,17 +912,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosRecursao3.pdf</t>
+          <t>ExerciciosIsabelle.pdf</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Recursao3</t>
+          <t>Exercicios Isabelle</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr"/>
@@ -935,17 +935,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosRecursao3_respostas.pdf</t>
+          <t>ExerciciosIsabelle2.pdf</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Recursao3 respostas</t>
+          <t>Exercicios Isabelle2</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr"/>
@@ -958,17 +958,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosIsabelle.pdf</t>
+          <t>ExerciciosLogicaTemporal.pdf</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Isabelle</t>
+          <t>Exercicios Logica Temporal</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr"/>
@@ -981,17 +981,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosIsabelle2.pdf</t>
+          <t>ExerciciosNusmv.pdf</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Isabelle2</t>
+          <t>Exercicios Nusmv</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosLogicaTemporal.pdf</t>
+          <t>FormalizacaoAlgoritmos_InvariantesLaco.pdf</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Logica Temporal</t>
+          <t>Formalizacao Algoritmos Invariantes Laco</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr"/>
@@ -1027,17 +1027,17 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosNusmv.pdf</t>
+          <t>FormalizacaoAlgoritmos_Recursao.pdf</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Nusmv</t>
+          <t>Formalizacao Algoritmos Recursao</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr"/>
@@ -1050,17 +1050,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>listas.thy</t>
+          <t>FormalizacaoAlgoritmos_Recursao2.pdf</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>listas</t>
+          <t>Formalizacao Algoritmos Recursao2</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
@@ -1073,17 +1073,17 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>LogicaDeHoare1_exercicios_respostas.pdf</t>
+          <t>FormalizacaoAlgoritmos_Recursao3.pdf</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>lista</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Logica De Hoare1 exercicios respostas</t>
+          <t>Formalizacao Algoritmos Recursao3</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr"/>
@@ -1096,17 +1096,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>arvores.thy</t>
+          <t>introducao.pdf</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>arvores</t>
+          <t>introducao</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr"/>
@@ -1119,17 +1119,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>classes_parte1.zip</t>
+          <t>LogicaDeHoare.pdf</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>classes parte1</t>
+          <t>Logica De Hoare</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
@@ -1142,17 +1142,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>classes_parte2.zip</t>
+          <t>LogicaDeHoare_exercicios_respostas.pdf</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>classes parte2</t>
+          <t>Logica De Hoare exercicios respostas</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
@@ -1165,17 +1165,17 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>colecoes_arrays.zip</t>
+          <t>LogicaDeHoare1_exercicios_respostas.pdf</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>colecoes arrays</t>
+          <t>Logica De Hoare1 exercicios respostas</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
@@ -1188,17 +1188,17 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>colecoes_conjuntos.zip</t>
+          <t>LogicaDeHoare2.pdf</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>colecoes conjuntos</t>
+          <t>Logica De Hoare2</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
@@ -1211,17 +1211,17 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>colecoes_sequences.zip</t>
+          <t>logicaPredicados_semantica.pdf</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>colecoes sequences</t>
+          <t>logica Predicados semantica</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr"/>
@@ -1234,17 +1234,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>exemplos.thy</t>
+          <t>logicaPredicados_sintaxe.pdf</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>exemplos</t>
+          <t>logica Predicados sintaxe</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
@@ -1257,17 +1257,17 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>exemplos.zip</t>
+          <t>logicaProposicional_semantica.pdf</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>exemplos</t>
+          <t>logica Proposicional semantica</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
@@ -1280,17 +1280,17 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>exercicios_arrays.zip</t>
+          <t>logicaProposicional_sintaxe.pdf</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>exercicios arrays</t>
+          <t>logica Proposicional sintaxe</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
@@ -1303,17 +1303,17 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>exercicios_conjuntos.zip</t>
+          <t>plano.pdf</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>exercicios conjuntos</t>
+          <t>plano</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>hoare.zip</t>
+          <t>ProvasIndutivas_EspecificaçõesRecursivas.pdf</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>hoare</t>
+          <t>Provas Indutivas Especificações Recursivas</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr"/>
@@ -1349,17 +1349,17 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>intro.thy</t>
+          <t>ProvasIndutivas_EspecificaçõesRecursivas_Arvores.pdf</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>intro</t>
+          <t>Provas Indutivas Especificações Recursivas Arvores</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
@@ -1372,17 +1372,17 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>introducao.zip</t>
+          <t>ProvasIndutivas_EspecificaçõesRecursivas_Listas.pdf</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>introducao</t>
+          <t>Provas Indutivas Especificações Recursivas Listas</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
@@ -1395,17 +1395,17 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>invariantes.zip</t>
+          <t>revisao.pdf</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>invariantes</t>
+          <t>revisao</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr"/>
@@ -1418,17 +1418,17 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>T1_2026_1.thy</t>
+          <t>revisao_p1.pdf</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>T1 2026 1</t>
+          <t>revisao p1</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr"/>
@@ -1441,17 +1441,17 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>terminacao.zip</t>
+          <t>revisao_p1_gabarito.pdf</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>terminacao</t>
+          <t>revisao p1 gabarito</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
@@ -1464,17 +1464,17 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>tiposindutivos.zip</t>
+          <t>t1_2026_1.pdf</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>código</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>tiposindutivos</t>
+          <t>t1 2026 1</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
@@ -1487,17 +1487,17 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Archive of Formal Proofs</t>
+          <t>t2_2026_1.pdf</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>Archive of Formal Proofs</t>
+          <t>t2 2026 1</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr"/>
@@ -1510,17 +1510,17 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>aws-encryption-sdk</t>
+          <t>verificacaomodelos.pdf</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>pdf</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>aws encryption sdk</t>
+          <t>verificacaomodelos</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr"/>
@@ -1533,17 +1533,17 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>eth2.0-dafny</t>
+          <t>arvores.thy</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>artigo</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>eth2.0 dafny</t>
+          <t>arvores</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr"/>
@@ -1556,17 +1556,17 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>ConjuntosIndutivos.pdf</t>
+          <t>classes_parte1.zip</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Conjuntos Indutivos</t>
+          <t>classes parte1</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr"/>
@@ -1579,17 +1579,17 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>CorrecaoTerminacao.pdf</t>
+          <t>classes_parte2.zip</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>Correcao Terminacao</t>
+          <t>classes parte2</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr"/>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosEspecificacao_respostas.pdf</t>
+          <t>colecoes_arrays.zip</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Especificacao respostas</t>
+          <t>colecoes arrays</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr"/>
@@ -1625,17 +1625,17 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>ExerciciosFormalizacaoAlgoritmosRecursao_respostas.pdf</t>
+          <t>colecoes_conjuntos.zip</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>Exercicios Formalizacao Algoritmos Recursao respostas</t>
+          <t>colecoes conjuntos</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr"/>
@@ -1648,17 +1648,17 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>FormalizacaoAlgoritmos_InvariantesLaco.pdf</t>
+          <t>colecoes_sequences.zip</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>Formalizacao Algoritmos Invariantes Laco</t>
+          <t>colecoes sequences</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr"/>
@@ -1671,17 +1671,17 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>FormalizacaoAlgoritmos_Recursao.pdf</t>
+          <t>exemplos.thy</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Formalizacao Algoritmos Recursao</t>
+          <t>exemplos</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr"/>
@@ -1694,17 +1694,17 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>FormalizacaoAlgoritmos_Recursao2.pdf</t>
+          <t>exemplos.zip</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>Formalizacao Algoritmos Recursao2</t>
+          <t>exemplos</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr"/>
@@ -1717,17 +1717,17 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>FormalizacaoAlgoritmos_Recursao3.pdf</t>
+          <t>exercicios_arrays.zip</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>Formalizacao Algoritmos Recursao3</t>
+          <t>exercicios arrays</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr"/>
@@ -1740,17 +1740,17 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>introducao.pdf</t>
+          <t>exercicios_conjuntos.zip</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>introducao</t>
+          <t>exercicios conjuntos</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr"/>
@@ -1763,17 +1763,17 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>LogicaDeHoare.pdf</t>
+          <t>hoare.zip</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>Logica De Hoare</t>
+          <t>hoare</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr"/>
@@ -1786,17 +1786,17 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>LogicaDeHoare_exercicios_respostas.pdf</t>
+          <t>intro.thy</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>Logica De Hoare exercicios respostas</t>
+          <t>intro</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
@@ -1809,17 +1809,17 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>LogicaDeHoare2.pdf</t>
+          <t>introducao.zip</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Logica De Hoare2</t>
+          <t>introducao</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr"/>
@@ -1832,17 +1832,17 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>logicaPredicados_semantica.pdf</t>
+          <t>invariantes.zip</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>logica Predicados semantica</t>
+          <t>invariantes</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr"/>
@@ -1855,17 +1855,17 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>logicaPredicados_sintaxe.pdf</t>
+          <t>listas.thy</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>logica Predicados sintaxe</t>
+          <t>listas</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr"/>
@@ -1878,17 +1878,17 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>logicaProposicional_semantica.pdf</t>
+          <t>provas.thy</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>logica Proposicional semantica</t>
+          <t>provas</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr"/>
@@ -1901,17 +1901,17 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>logicaProposicional_sintaxe.pdf</t>
+          <t>T1_2026_1.thy</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>logica Proposicional sintaxe</t>
+          <t>T1 2026 1</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr"/>
@@ -1924,17 +1924,17 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>plano.pdf</t>
+          <t>terminacao.zip</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>plano</t>
+          <t>terminacao</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr"/>
@@ -1947,17 +1947,17 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>revisao.pdf</t>
+          <t>tiposindutivos.zip</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>código</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>revisao</t>
+          <t>tiposindutivos</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr"/>
@@ -1970,17 +1970,17 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>t1_2026_1.pdf</t>
+          <t>Archive of Formal Proofs</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>link</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>t1 2026 1</t>
+          <t>Archive of Formal Proofs</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr"/>
@@ -1993,17 +1993,17 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>t2_2026_1.pdf</t>
+          <t>aws-encryption-sdk</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>github-repo</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>t2 2026 1</t>
+          <t>aws encryption sdk</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr"/>
@@ -2016,17 +2016,17 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>verificacaomodelos.pdf</t>
+          <t>eth2.0-dafny</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>github-repo</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>verificacaomodelos</t>
+          <t>eth2.0 dafny</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr"/>

</xml_diff>